<commit_message>
finished up to figure 4
</commit_message>
<xml_diff>
--- a/sheets/fig2.xlsx
+++ b/sheets/fig2.xlsx
@@ -5,16 +5,16 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Neu" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="main.smu" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="cs_g" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="cs_E" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="cs_FAT" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="es" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="noise" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="Neu" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="main.smu" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="cs_g" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="cs_E" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="cs_FAT" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="es" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="noise" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -597,7 +597,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Cambria Math"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1220,663 +1220,663 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="28" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="27" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="27" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="21" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="29" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="29" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="30" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="30" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="31" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="31" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="33" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="33" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="34" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="34" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="35" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="35" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="36" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="36" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="37" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="37" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="42" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="42" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="43" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="46" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="44" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="40" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="32" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="41" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="47" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="45" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="51" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="51" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="52" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="52" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="51" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="51" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="53" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="53" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="54" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="54" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="55" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="55" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="56" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="56" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="57" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="57" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="58" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="58" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="59" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="59" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="60" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="60" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="61" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="61" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="62" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="62" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="63" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="63" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="64" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="64" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="65" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="65" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="66" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="66" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="67" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="67" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="35" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="35" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="68" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="68" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="69" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="69" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="47" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="47" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="43" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="43" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="44" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="44" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2149,7 +2149,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -2166,7 +2166,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -2319,13 +2319,13 @@
       <xdr:col>36</xdr:col>
       <xdr:colOff>93240</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4680</xdr:rowOff>
+      <xdr:rowOff>15480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>39</xdr:col>
-      <xdr:colOff>45360</xdr:colOff>
+      <xdr:colOff>45000</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>103320</xdr:rowOff>
+      <xdr:rowOff>113760</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2334,8 +2334,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="20979720" y="928440"/>
-          <a:ext cx="2400120" cy="279720"/>
+          <a:off x="16656120" y="928440"/>
+          <a:ext cx="1892880" cy="279360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2390,13 +2390,119 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:JX62"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="9.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.45"/>
@@ -2610,7 +2716,7 @@
       <c r="AF1" s="4"/>
       <c r="AG1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E2" s="5" t="s">
         <v>3</v>
       </c>
@@ -2649,7 +2755,7 @@
       <c r="AF2" s="8"/>
       <c r="AG2" s="8"/>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -2750,7 +2856,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="str">
         <f aca="false">Neu!B4</f>
         <v>cell</v>
@@ -2796,7 +2902,7 @@
       <c r="AF4" s="24"/>
       <c r="AG4" s="25"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="n">
         <f aca="false">Neu!B5</f>
         <v>0</v>
@@ -2834,7 +2940,7 @@
       <c r="AF5" s="27"/>
       <c r="AG5" s="20"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="n">
         <f aca="false">Neu!B6</f>
         <v>0</v>
@@ -2872,7 +2978,7 @@
       <c r="AF6" s="27"/>
       <c r="AG6" s="20"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="n">
         <f aca="false">Neu!B7</f>
         <v>0</v>
@@ -2910,7 +3016,7 @@
       <c r="AF7" s="27"/>
       <c r="AG7" s="20"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="n">
         <f aca="false">Neu!B8</f>
         <v>0</v>
@@ -2948,7 +3054,7 @@
       <c r="AF8" s="27"/>
       <c r="AG8" s="20"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="n">
         <f aca="false">Neu!B9</f>
         <v>0</v>
@@ -2986,7 +3092,7 @@
       <c r="AF9" s="27"/>
       <c r="AG9" s="20"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="n">
         <f aca="false">Neu!B10</f>
         <v>0</v>
@@ -3024,7 +3130,7 @@
       <c r="AF10" s="27"/>
       <c r="AG10" s="20"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="n">
         <f aca="false">Neu!B11</f>
         <v>0</v>
@@ -3062,7 +3168,7 @@
       <c r="AF11" s="27"/>
       <c r="AG11" s="20"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="n">
         <f aca="false">Neu!B12</f>
         <v>0</v>
@@ -3100,7 +3206,7 @@
       <c r="AF12" s="27"/>
       <c r="AG12" s="20"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="n">
         <f aca="false">Neu!B13</f>
         <v>0</v>
@@ -3138,7 +3244,7 @@
       <c r="AF13" s="27"/>
       <c r="AG13" s="20"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="n">
         <f aca="false">Neu!B14</f>
         <v>0</v>
@@ -3176,7 +3282,7 @@
       <c r="AF14" s="27"/>
       <c r="AG14" s="20"/>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="n">
         <f aca="false">Neu!B15</f>
         <v>0</v>
@@ -3214,7 +3320,7 @@
       <c r="AF15" s="27"/>
       <c r="AG15" s="20"/>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="n">
         <f aca="false">Neu!B16</f>
         <v>0</v>
@@ -3252,7 +3358,7 @@
       <c r="AF16" s="27"/>
       <c r="AG16" s="20"/>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="n">
         <f aca="false">Neu!B17</f>
         <v>0</v>
@@ -3290,7 +3396,7 @@
       <c r="AF17" s="27"/>
       <c r="AG17" s="20"/>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="n">
         <f aca="false">Neu!B18</f>
         <v>0</v>
@@ -3328,7 +3434,7 @@
       <c r="AF18" s="27"/>
       <c r="AG18" s="20"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="n">
         <f aca="false">Neu!B19</f>
         <v>0</v>
@@ -3366,7 +3472,7 @@
       <c r="AF19" s="27"/>
       <c r="AG19" s="20"/>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="n">
         <f aca="false">Neu!B20</f>
         <v>0</v>
@@ -3404,7 +3510,7 @@
       <c r="AF20" s="27"/>
       <c r="AG20" s="20"/>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="n">
         <f aca="false">Neu!B21</f>
         <v>0</v>
@@ -3442,7 +3548,7 @@
       <c r="AF21" s="27"/>
       <c r="AG21" s="20"/>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="n">
         <f aca="false">Neu!B22</f>
         <v>0</v>
@@ -3480,7 +3586,7 @@
       <c r="AF22" s="27"/>
       <c r="AG22" s="20"/>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="n">
         <f aca="false">Neu!B23</f>
         <v>0</v>
@@ -3518,7 +3624,7 @@
       <c r="AF23" s="27"/>
       <c r="AG23" s="20"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="n">
         <f aca="false">Neu!B24</f>
         <v>0</v>
@@ -3942,7 +4048,7 @@
       <c r="EG28" s="34"/>
       <c r="EH28" s="34"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D29" s="35" t="s">
         <v>26</v>
       </c>
@@ -3981,7 +4087,7 @@
       <c r="EH29" s="34"/>
       <c r="HO29" s="34"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D30" s="36" t="s">
         <v>7</v>
       </c>
@@ -4144,7 +4250,7 @@
       <c r="DV30" s="34"/>
       <c r="HO30" s="34"/>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D31" s="41"/>
       <c r="E31" s="42"/>
       <c r="F31" s="27"/>
@@ -4211,7 +4317,7 @@
       <c r="DV31" s="34"/>
       <c r="HO31" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="45" t="n">
         <f aca="false">Neu!$B5</f>
         <v>0</v>
@@ -4286,7 +4392,7 @@
       <c r="DU32" s="34"/>
       <c r="DV32" s="34"/>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D33" s="45" t="n">
         <f aca="false">Neu!$B6</f>
         <v>0</v>
@@ -4361,7 +4467,7 @@
       <c r="DU33" s="34"/>
       <c r="DV33" s="34"/>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D34" s="45" t="n">
         <f aca="false">Neu!$B7</f>
         <v>0</v>
@@ -4427,7 +4533,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D35" s="45" t="n">
         <f aca="false">Neu!$B8</f>
         <v>0</v>
@@ -4493,7 +4599,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D36" s="45" t="n">
         <f aca="false">Neu!$B9</f>
         <v>0</v>
@@ -4559,7 +4665,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D37" s="45" t="n">
         <f aca="false">Neu!$B10</f>
         <v>0</v>
@@ -4625,7 +4731,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D38" s="45" t="n">
         <f aca="false">Neu!$B11</f>
         <v>0</v>
@@ -4691,7 +4797,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D39" s="45" t="n">
         <f aca="false">Neu!$B12</f>
         <v>0</v>
@@ -4757,7 +4863,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D40" s="45" t="n">
         <f aca="false">Neu!$B13</f>
         <v>0</v>
@@ -4823,7 +4929,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D41" s="45" t="n">
         <f aca="false">Neu!$B14</f>
         <v>0</v>
@@ -4889,7 +4995,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D42" s="45" t="n">
         <f aca="false">Neu!$B15</f>
         <v>0</v>
@@ -4955,7 +5061,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D43" s="45" t="n">
         <f aca="false">Neu!$B16</f>
         <v>0</v>
@@ -5021,7 +5127,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D44" s="45" t="n">
         <f aca="false">Neu!$B17</f>
         <v>0</v>
@@ -5087,7 +5193,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D45" s="45" t="n">
         <f aca="false">Neu!$B18</f>
         <v>0</v>
@@ -5153,7 +5259,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D46" s="45" t="n">
         <f aca="false">Neu!$B19</f>
         <v>0</v>
@@ -5219,7 +5325,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D47" s="45" t="n">
         <f aca="false">Neu!$B20</f>
         <v>0</v>
@@ -5285,7 +5391,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D48" s="45" t="n">
         <f aca="false">Neu!$B21</f>
         <v>0</v>
@@ -5349,7 +5455,7 @@
       </c>
       <c r="BE48" s="42"/>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D49" s="45" t="n">
         <f aca="false">Neu!$B22</f>
         <v>0</v>
@@ -5413,7 +5519,7 @@
       </c>
       <c r="BE49" s="42"/>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D50" s="45" t="n">
         <f aca="false">Neu!$B23</f>
         <v>0</v>
@@ -5477,7 +5583,7 @@
       </c>
       <c r="BE50" s="42"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D51" s="46" t="n">
         <f aca="false">Neu!$B24</f>
         <v>0</v>
@@ -5832,12 +5938,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z87"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="34" width="8.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="34" width="10.54"/>
@@ -6052,7 +6158,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="59" t="s">
         <v>115</v>
       </c>
@@ -6066,7 +6172,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="61" t="s">
         <v>119</v>
       </c>
@@ -6597,7 +6703,7 @@
       <c r="Y22" s="27"/>
       <c r="Z22" s="20"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="70"/>
       <c r="B23" s="71"/>
       <c r="C23" s="32"/>
@@ -7391,12 +7497,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AD76"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="75" width="4.18"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="75" width="9.18"/>
@@ -7404,7 +7510,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="24" style="75" width="9.18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="76"/>
       <c r="B1" s="76"/>
       <c r="C1" s="77" t="s">
@@ -7431,7 +7537,7 @@
       <c r="V1" s="77"/>
       <c r="W1" s="77"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="76"/>
       <c r="B2" s="76"/>
       <c r="C2" s="78" t="str">
@@ -10036,12 +10142,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AD76"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="75" width="4.18"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="75" width="9.18"/>
@@ -10049,7 +10155,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="24" style="75" width="9.18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="76"/>
       <c r="B1" s="76"/>
       <c r="C1" s="77" t="s">
@@ -10076,7 +10182,7 @@
       <c r="V1" s="77"/>
       <c r="W1" s="77"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="76"/>
       <c r="B2" s="76"/>
       <c r="C2" s="78" t="str">
@@ -12713,12 +12819,12 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AL229"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="75" width="4.18"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="75" width="9.18"/>
@@ -12736,7 +12842,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="37" style="75" width="9.18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="76"/>
       <c r="B1" s="76"/>
       <c r="C1" s="127" t="s">
@@ -12781,7 +12887,7 @@
       </c>
       <c r="AJ1" s="128"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="76"/>
       <c r="B2" s="76"/>
       <c r="C2" s="78" t="str">
@@ -15552,7 +15658,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4CDA65FC-5416-43A0-BDD2-B2EFBC6D3811}</x14:id>
+          <x14:id>{1EC91B22-C491-428A-A9C4-BB6CDD12B070}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -15581,7 +15687,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4CDA65FC-5416-43A0-BDD2-B2EFBC6D3811}">
+          <x14:cfRule type="dataBar" id="{1EC91B22-C491-428A-A9C4-BB6CDD12B070}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="automatic" gradient="false">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -15598,12 +15704,12 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.18"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.18"/>
@@ -15612,7 +15718,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="26" style="1" width="9.18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="139"/>
       <c r="B1" s="139"/>
       <c r="C1" s="140" t="s">
@@ -15633,7 +15739,7 @@
       <c r="P1" s="140"/>
       <c r="Q1" s="140"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="139"/>
       <c r="B2" s="139"/>
       <c r="C2" s="141" t="str">
@@ -16985,12 +17091,12 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="162" width="35.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="163" width="10.82"/>

</xml_diff>